<commit_message>
Refactor document structure and update workspace configuration
- Changed the type of multiple documents from "pracovni_balicek" to "cinnost" and updated their metadata accordingly for better clarity and organization.
- Adjusted dataview queries across various documents to ensure they accurately reflect the new structure and improve data retrieval.
- Updated the workspace configuration to enhance the recently opened files list, ensuring it reflects the current document context and improves navigation.
</commit_message>
<xml_diff>
--- a/00_Podklady/(šablona) Příloha_1_Matice_informačního_managementu_(RACI).xlsx
+++ b/00_Podklady/(šablona) Příloha_1_Matice_informačního_managementu_(RACI).xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liftrock.sharepoint.com/sites/BIMServices/Sdilene dokumenty/General/04_Šablony/02_Šablony plánu realizace BIM/Obecné/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liftrock.sharepoint.com/sites/BIMServices/Sdilene dokumenty/General/01_Zakázky/ZAK_2023_060 ŘSD Plzeň CDE koordinátor/knowledge_base/00_Podklady/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="273" documentId="8_{1A589C59-B8ED-4025-8D09-CAE49E68BD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDAFB3EC-F676-40A1-B9DF-2FF7C11FC40B}"/>
@@ -2477,26 +2477,11 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="7" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="7" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2517,6 +2502,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="7" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="7" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2869,36 +2869,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:90" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="121" t="s">
         <v>342</v>
       </c>
-      <c r="B1" s="111" t="s">
+      <c r="B1" s="109" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="111" t="s">
+      <c r="C1" s="109" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="111" t="s">
+      <c r="D1" s="109" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="117" t="s">
+      <c r="E1" s="112" t="s">
         <v>349</v>
       </c>
-      <c r="F1" s="118"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="120" t="s">
+      <c r="F1" s="113"/>
+      <c r="G1" s="114"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="115" t="s">
         <v>350</v>
       </c>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="122"/>
-    </row>
-    <row r="2" spans="1:90" s="23" customFormat="1" ht="148.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="110"/>
-      <c r="B2" s="112"/>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
+      <c r="J1" s="116"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="117"/>
+    </row>
+    <row r="2" spans="1:90" s="23" customFormat="1" ht="137.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="122"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
       <c r="E2" s="13" t="s">
         <v>336</v>
       </c>
@@ -2908,7 +2908,7 @@
       <c r="G2" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="H2" s="116"/>
+      <c r="H2" s="111"/>
       <c r="I2" s="14" t="s">
         <v>352</v>
       </c>
@@ -4070,7 +4070,7 @@
       <c r="B21" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="113" t="s">
+      <c r="C21" s="118" t="s">
         <v>430</v>
       </c>
       <c r="D21" s="51" t="s">
@@ -4100,7 +4100,7 @@
       <c r="B22" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="115"/>
+      <c r="C22" s="119"/>
       <c r="D22" s="51" t="s">
         <v>363</v>
       </c>
@@ -4128,7 +4128,7 @@
       <c r="B23" s="49" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="115"/>
+      <c r="C23" s="119"/>
       <c r="D23" s="51" t="s">
         <v>363</v>
       </c>
@@ -4156,7 +4156,7 @@
       <c r="B24" s="49" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="115"/>
+      <c r="C24" s="119"/>
       <c r="D24" s="51" t="s">
         <v>363</v>
       </c>
@@ -4184,7 +4184,7 @@
       <c r="B25" s="49" t="s">
         <v>55</v>
       </c>
-      <c r="C25" s="115"/>
+      <c r="C25" s="119"/>
       <c r="D25" s="51" t="s">
         <v>363</v>
       </c>
@@ -4212,7 +4212,7 @@
       <c r="B26" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="C26" s="114"/>
+      <c r="C26" s="120"/>
       <c r="D26" s="51" t="s">
         <v>58</v>
       </c>
@@ -4580,7 +4580,7 @@
       <c r="B31" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="113" t="s">
+      <c r="C31" s="118" t="s">
         <v>432</v>
       </c>
       <c r="D31" s="51" t="s">
@@ -4612,7 +4612,7 @@
       <c r="B32" s="49" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="115"/>
+      <c r="C32" s="119"/>
       <c r="D32" s="51" t="s">
         <v>368</v>
       </c>
@@ -4642,7 +4642,7 @@
       <c r="B33" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="115"/>
+      <c r="C33" s="119"/>
       <c r="D33" s="51" t="s">
         <v>369</v>
       </c>
@@ -4672,7 +4672,7 @@
       <c r="B34" s="49" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="115"/>
+      <c r="C34" s="119"/>
       <c r="D34" s="51" t="s">
         <v>370</v>
       </c>
@@ -4702,7 +4702,7 @@
       <c r="B35" s="49" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="115"/>
+      <c r="C35" s="119"/>
       <c r="D35" s="51" t="s">
         <v>371</v>
       </c>
@@ -4732,7 +4732,7 @@
       <c r="B36" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="C36" s="114"/>
+      <c r="C36" s="120"/>
       <c r="D36" s="51" t="s">
         <v>372</v>
       </c>
@@ -5230,7 +5230,7 @@
       <c r="B45" s="49" t="s">
         <v>98</v>
       </c>
-      <c r="C45" s="113" t="s">
+      <c r="C45" s="118" t="s">
         <v>99</v>
       </c>
       <c r="D45" s="51" t="s">
@@ -5262,7 +5262,7 @@
       <c r="B46" s="49" t="s">
         <v>101</v>
       </c>
-      <c r="C46" s="115"/>
+      <c r="C46" s="119"/>
       <c r="D46" s="51" t="s">
         <v>377</v>
       </c>
@@ -5292,7 +5292,7 @@
       <c r="B47" s="49" t="s">
         <v>103</v>
       </c>
-      <c r="C47" s="115"/>
+      <c r="C47" s="119"/>
       <c r="D47" s="51" t="s">
         <v>377</v>
       </c>
@@ -5322,7 +5322,7 @@
       <c r="B48" s="49" t="s">
         <v>105</v>
       </c>
-      <c r="C48" s="115"/>
+      <c r="C48" s="119"/>
       <c r="D48" s="51" t="s">
         <v>377</v>
       </c>
@@ -5352,7 +5352,7 @@
       <c r="B49" s="49" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="115"/>
+      <c r="C49" s="119"/>
       <c r="D49" s="51" t="s">
         <v>377</v>
       </c>
@@ -5382,7 +5382,7 @@
       <c r="B50" s="49" t="s">
         <v>109</v>
       </c>
-      <c r="C50" s="115"/>
+      <c r="C50" s="119"/>
       <c r="D50" s="51" t="s">
         <v>377</v>
       </c>
@@ -5412,7 +5412,7 @@
       <c r="B51" s="49" t="s">
         <v>111</v>
       </c>
-      <c r="C51" s="115"/>
+      <c r="C51" s="119"/>
       <c r="D51" s="51" t="s">
         <v>377</v>
       </c>
@@ -5442,7 +5442,7 @@
       <c r="B52" s="49" t="s">
         <v>113</v>
       </c>
-      <c r="C52" s="115"/>
+      <c r="C52" s="119"/>
       <c r="D52" s="51" t="s">
         <v>377</v>
       </c>
@@ -5472,7 +5472,7 @@
       <c r="B53" s="49" t="s">
         <v>115</v>
       </c>
-      <c r="C53" s="114"/>
+      <c r="C53" s="120"/>
       <c r="D53" s="51" t="s">
         <v>58</v>
       </c>
@@ -5989,7 +5989,7 @@
       <c r="CK61" s="21"/>
       <c r="CL61" s="21"/>
     </row>
-    <row r="62" spans="1:90" ht="26.4" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:90" ht="39.6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A62" s="48" t="s">
         <v>130</v>
       </c>
@@ -6240,7 +6240,7 @@
       <c r="CK65" s="21"/>
       <c r="CL65" s="21"/>
     </row>
-    <row r="66" spans="1:90" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:90" ht="26.4" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A66" s="48" t="s">
         <v>138</v>
       </c>
@@ -6498,7 +6498,7 @@
       <c r="B70" s="49" t="s">
         <v>439</v>
       </c>
-      <c r="C70" s="113" t="s">
+      <c r="C70" s="118" t="s">
         <v>149</v>
       </c>
       <c r="D70" s="51" t="s">
@@ -6521,7 +6521,7 @@
       <c r="B71" s="49" t="s">
         <v>151</v>
       </c>
-      <c r="C71" s="115"/>
+      <c r="C71" s="119"/>
       <c r="D71" s="51" t="s">
         <v>385</v>
       </c>
@@ -6542,7 +6542,7 @@
       <c r="B72" s="49" t="s">
         <v>153</v>
       </c>
-      <c r="C72" s="115"/>
+      <c r="C72" s="119"/>
       <c r="D72" s="51" t="s">
         <v>385</v>
       </c>
@@ -6563,7 +6563,7 @@
       <c r="B73" s="49" t="s">
         <v>155</v>
       </c>
-      <c r="C73" s="114"/>
+      <c r="C73" s="120"/>
       <c r="D73" s="51" t="s">
         <v>385</v>
       </c>
@@ -6688,7 +6688,7 @@
       <c r="B75" s="49" t="s">
         <v>159</v>
       </c>
-      <c r="C75" s="113" t="s">
+      <c r="C75" s="118" t="s">
         <v>160</v>
       </c>
       <c r="D75" s="51" t="s">
@@ -6722,7 +6722,7 @@
       <c r="B76" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="C76" s="115"/>
+      <c r="C76" s="119"/>
       <c r="D76" s="51" t="s">
         <v>58</v>
       </c>
@@ -6754,7 +6754,7 @@
       <c r="B77" s="49" t="s">
         <v>164</v>
       </c>
-      <c r="C77" s="114"/>
+      <c r="C77" s="120"/>
       <c r="D77" s="51" t="s">
         <v>58</v>
       </c>
@@ -6989,7 +6989,7 @@
       <c r="B80" s="49" t="s">
         <v>440</v>
       </c>
-      <c r="C80" s="113" t="s">
+      <c r="C80" s="118" t="s">
         <v>170</v>
       </c>
       <c r="D80" s="51" t="s">
@@ -7018,7 +7018,7 @@
       <c r="B81" s="49" t="s">
         <v>172</v>
       </c>
-      <c r="C81" s="115"/>
+      <c r="C81" s="119"/>
       <c r="D81" s="51" t="s">
         <v>388</v>
       </c>
@@ -7045,7 +7045,7 @@
       <c r="B82" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="C82" s="115"/>
+      <c r="C82" s="119"/>
       <c r="D82" s="51" t="s">
         <v>389</v>
       </c>
@@ -7072,7 +7072,7 @@
       <c r="B83" s="49" t="s">
         <v>176</v>
       </c>
-      <c r="C83" s="115"/>
+      <c r="C83" s="119"/>
       <c r="D83" s="51" t="s">
         <v>390</v>
       </c>
@@ -7099,7 +7099,7 @@
       <c r="B84" s="83" t="s">
         <v>178</v>
       </c>
-      <c r="C84" s="115"/>
+      <c r="C84" s="119"/>
       <c r="D84" s="51" t="s">
         <v>391</v>
       </c>
@@ -7126,7 +7126,7 @@
       <c r="B85" s="49" t="s">
         <v>180</v>
       </c>
-      <c r="C85" s="115"/>
+      <c r="C85" s="119"/>
       <c r="D85" s="51" t="s">
         <v>392</v>
       </c>
@@ -7153,7 +7153,7 @@
       <c r="B86" s="49" t="s">
         <v>182</v>
       </c>
-      <c r="C86" s="114"/>
+      <c r="C86" s="120"/>
       <c r="D86" s="51" t="s">
         <v>393</v>
       </c>
@@ -7282,7 +7282,7 @@
       <c r="B88" s="49" t="s">
         <v>186</v>
       </c>
-      <c r="C88" s="113" t="s">
+      <c r="C88" s="118" t="s">
         <v>187</v>
       </c>
       <c r="D88" s="51" t="s">
@@ -7307,7 +7307,7 @@
       <c r="B89" s="49" t="s">
         <v>189</v>
       </c>
-      <c r="C89" s="114"/>
+      <c r="C89" s="120"/>
       <c r="D89" s="51" t="s">
         <v>58</v>
       </c>
@@ -7430,7 +7430,7 @@
       <c r="B91" s="49" t="s">
         <v>191</v>
       </c>
-      <c r="C91" s="113" t="s">
+      <c r="C91" s="118" t="s">
         <v>193</v>
       </c>
       <c r="D91" s="51" t="s">
@@ -7453,7 +7453,7 @@
       <c r="B92" s="49" t="s">
         <v>195</v>
       </c>
-      <c r="C92" s="115"/>
+      <c r="C92" s="119"/>
       <c r="D92" s="51" t="s">
         <v>396</v>
       </c>
@@ -7474,7 +7474,7 @@
       <c r="B93" s="49" t="s">
         <v>197</v>
       </c>
-      <c r="C93" s="115"/>
+      <c r="C93" s="119"/>
       <c r="D93" s="51" t="s">
         <v>397</v>
       </c>
@@ -7495,7 +7495,7 @@
       <c r="B94" s="49" t="s">
         <v>199</v>
       </c>
-      <c r="C94" s="115"/>
+      <c r="C94" s="119"/>
       <c r="D94" s="87" t="s">
         <v>398</v>
       </c>
@@ -7516,7 +7516,7 @@
       <c r="B95" s="49" t="s">
         <v>201</v>
       </c>
-      <c r="C95" s="115"/>
+      <c r="C95" s="119"/>
       <c r="D95" s="87" t="s">
         <v>399</v>
       </c>
@@ -7537,7 +7537,7 @@
       <c r="B96" s="49" t="s">
         <v>203</v>
       </c>
-      <c r="C96" s="114"/>
+      <c r="C96" s="120"/>
       <c r="D96" s="87" t="s">
         <v>400</v>
       </c>
@@ -7660,7 +7660,7 @@
       <c r="B98" s="49" t="s">
         <v>207</v>
       </c>
-      <c r="C98" s="113" t="s">
+      <c r="C98" s="118" t="s">
         <v>208</v>
       </c>
       <c r="D98" s="51" t="s">
@@ -7683,7 +7683,7 @@
       <c r="B99" s="49" t="s">
         <v>210</v>
       </c>
-      <c r="C99" s="114"/>
+      <c r="C99" s="120"/>
       <c r="D99" s="51" t="s">
         <v>401</v>
       </c>
@@ -7810,7 +7810,7 @@
       <c r="B101" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="C101" s="113" t="s">
+      <c r="C101" s="118" t="s">
         <v>216</v>
       </c>
       <c r="D101" s="51" t="s">
@@ -7835,7 +7835,7 @@
       <c r="B102" s="49" t="s">
         <v>218</v>
       </c>
-      <c r="C102" s="115"/>
+      <c r="C102" s="119"/>
       <c r="D102" s="51" t="s">
         <v>402</v>
       </c>
@@ -7858,7 +7858,7 @@
       <c r="B103" s="49" t="s">
         <v>220</v>
       </c>
-      <c r="C103" s="115"/>
+      <c r="C103" s="119"/>
       <c r="D103" s="51" t="s">
         <v>402</v>
       </c>
@@ -7881,7 +7881,7 @@
       <c r="B104" s="49" t="s">
         <v>222</v>
       </c>
-      <c r="C104" s="114"/>
+      <c r="C104" s="120"/>
       <c r="D104" s="51" t="s">
         <v>402</v>
       </c>
@@ -8012,7 +8012,7 @@
       <c r="B106" s="49" t="s">
         <v>226</v>
       </c>
-      <c r="C106" s="113" t="s">
+      <c r="C106" s="118" t="s">
         <v>443</v>
       </c>
       <c r="D106" s="51" t="s">
@@ -8039,7 +8039,7 @@
       <c r="B107" s="49" t="s">
         <v>228</v>
       </c>
-      <c r="C107" s="115"/>
+      <c r="C107" s="119"/>
       <c r="D107" s="51" t="s">
         <v>403</v>
       </c>
@@ -8064,7 +8064,7 @@
       <c r="B108" s="49" t="s">
         <v>230</v>
       </c>
-      <c r="C108" s="115"/>
+      <c r="C108" s="119"/>
       <c r="D108" s="51" t="s">
         <v>403</v>
       </c>
@@ -8089,7 +8089,7 @@
       <c r="B109" s="49" t="s">
         <v>232</v>
       </c>
-      <c r="C109" s="115"/>
+      <c r="C109" s="119"/>
       <c r="D109" s="51" t="s">
         <v>403</v>
       </c>
@@ -8114,7 +8114,7 @@
       <c r="B110" s="49" t="s">
         <v>441</v>
       </c>
-      <c r="C110" s="115"/>
+      <c r="C110" s="119"/>
       <c r="D110" s="51" t="s">
         <v>403</v>
       </c>
@@ -8139,7 +8139,7 @@
       <c r="B111" s="49" t="s">
         <v>235</v>
       </c>
-      <c r="C111" s="115"/>
+      <c r="C111" s="119"/>
       <c r="D111" s="51" t="s">
         <v>403</v>
       </c>
@@ -8164,7 +8164,7 @@
       <c r="B112" s="49" t="s">
         <v>442</v>
       </c>
-      <c r="C112" s="115"/>
+      <c r="C112" s="119"/>
       <c r="D112" s="51" t="s">
         <v>58</v>
       </c>
@@ -8189,7 +8189,7 @@
       <c r="B113" s="49" t="s">
         <v>238</v>
       </c>
-      <c r="C113" s="114"/>
+      <c r="C113" s="120"/>
       <c r="D113" s="51" t="s">
         <v>58</v>
       </c>
@@ -8316,7 +8316,7 @@
       <c r="B115" s="49" t="s">
         <v>242</v>
       </c>
-      <c r="C115" s="113" t="s">
+      <c r="C115" s="118" t="s">
         <v>444</v>
       </c>
       <c r="D115" s="51" t="s">
@@ -8334,14 +8334,14 @@
       <c r="K115" s="53"/>
       <c r="L115" s="57"/>
     </row>
-    <row r="116" spans="1:90" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:90" ht="26.4" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A116" s="48" t="s">
         <v>243</v>
       </c>
       <c r="B116" s="49" t="s">
         <v>244</v>
       </c>
-      <c r="C116" s="115"/>
+      <c r="C116" s="119"/>
       <c r="D116" s="51" t="s">
         <v>404</v>
       </c>
@@ -8364,7 +8364,7 @@
       <c r="B117" s="49" t="s">
         <v>230</v>
       </c>
-      <c r="C117" s="115"/>
+      <c r="C117" s="119"/>
       <c r="D117" s="51" t="s">
         <v>404</v>
       </c>
@@ -8387,7 +8387,7 @@
       <c r="B118" s="49" t="s">
         <v>232</v>
       </c>
-      <c r="C118" s="115"/>
+      <c r="C118" s="119"/>
       <c r="D118" s="51" t="s">
         <v>404</v>
       </c>
@@ -8410,7 +8410,7 @@
       <c r="B119" s="49" t="s">
         <v>441</v>
       </c>
-      <c r="C119" s="115"/>
+      <c r="C119" s="119"/>
       <c r="D119" s="51" t="s">
         <v>404</v>
       </c>
@@ -8433,7 +8433,7 @@
       <c r="B120" s="49" t="s">
         <v>249</v>
       </c>
-      <c r="C120" s="115"/>
+      <c r="C120" s="119"/>
       <c r="D120" s="51" t="s">
         <v>404</v>
       </c>
@@ -8456,7 +8456,7 @@
       <c r="B121" s="49" t="s">
         <v>442</v>
       </c>
-      <c r="C121" s="115"/>
+      <c r="C121" s="119"/>
       <c r="D121" s="51" t="s">
         <v>58</v>
       </c>
@@ -8479,7 +8479,7 @@
       <c r="B122" s="49" t="s">
         <v>252</v>
       </c>
-      <c r="C122" s="114"/>
+      <c r="C122" s="120"/>
       <c r="D122" s="51" t="s">
         <v>58</v>
       </c>
@@ -8706,7 +8706,7 @@
       <c r="B125" s="49" t="s">
         <v>257</v>
       </c>
-      <c r="C125" s="113" t="s">
+      <c r="C125" s="118" t="s">
         <v>258</v>
       </c>
       <c r="D125" s="51" t="s">
@@ -8731,7 +8731,7 @@
       <c r="B126" s="49" t="s">
         <v>260</v>
       </c>
-      <c r="C126" s="115"/>
+      <c r="C126" s="119"/>
       <c r="D126" s="51" t="s">
         <v>406</v>
       </c>
@@ -8754,7 +8754,7 @@
       <c r="B127" s="49" t="s">
         <v>262</v>
       </c>
-      <c r="C127" s="115"/>
+      <c r="C127" s="119"/>
       <c r="D127" s="51" t="s">
         <v>406</v>
       </c>
@@ -8777,7 +8777,7 @@
       <c r="B128" s="49" t="s">
         <v>264</v>
       </c>
-      <c r="C128" s="114"/>
+      <c r="C128" s="120"/>
       <c r="D128" s="51" t="s">
         <v>406</v>
       </c>
@@ -8902,7 +8902,7 @@
       <c r="B130" s="49" t="s">
         <v>268</v>
       </c>
-      <c r="C130" s="113" t="s">
+      <c r="C130" s="118" t="s">
         <v>269</v>
       </c>
       <c r="D130" s="51" t="s">
@@ -8929,7 +8929,7 @@
       <c r="B131" s="49" t="s">
         <v>271</v>
       </c>
-      <c r="C131" s="115"/>
+      <c r="C131" s="119"/>
       <c r="D131" s="51" t="s">
         <v>407</v>
       </c>
@@ -8954,7 +8954,7 @@
       <c r="B132" s="49" t="s">
         <v>445</v>
       </c>
-      <c r="C132" s="115"/>
+      <c r="C132" s="119"/>
       <c r="D132" s="51" t="s">
         <v>407</v>
       </c>
@@ -8979,7 +8979,7 @@
       <c r="B133" s="49" t="s">
         <v>446</v>
       </c>
-      <c r="C133" s="115"/>
+      <c r="C133" s="119"/>
       <c r="D133" s="51" t="s">
         <v>407</v>
       </c>
@@ -9004,7 +9004,7 @@
       <c r="B134" s="49" t="s">
         <v>275</v>
       </c>
-      <c r="C134" s="115"/>
+      <c r="C134" s="119"/>
       <c r="D134" s="51" t="s">
         <v>407</v>
       </c>
@@ -9029,7 +9029,7 @@
       <c r="B135" s="49" t="s">
         <v>277</v>
       </c>
-      <c r="C135" s="114"/>
+      <c r="C135" s="120"/>
       <c r="D135" s="51" t="s">
         <v>407</v>
       </c>
@@ -9160,7 +9160,7 @@
       <c r="B137" s="49" t="s">
         <v>281</v>
       </c>
-      <c r="C137" s="113" t="s">
+      <c r="C137" s="118" t="s">
         <v>282</v>
       </c>
       <c r="D137" s="51" t="s">
@@ -9189,7 +9189,7 @@
       <c r="B138" s="49" t="s">
         <v>284</v>
       </c>
-      <c r="C138" s="115"/>
+      <c r="C138" s="119"/>
       <c r="D138" s="51" t="s">
         <v>408</v>
       </c>
@@ -9214,7 +9214,7 @@
       <c r="B139" s="49" t="s">
         <v>286</v>
       </c>
-      <c r="C139" s="115"/>
+      <c r="C139" s="119"/>
       <c r="D139" s="51" t="s">
         <v>408</v>
       </c>
@@ -9239,7 +9239,7 @@
       <c r="B140" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C140" s="114"/>
+      <c r="C140" s="120"/>
       <c r="D140" s="51" t="s">
         <v>408</v>
       </c>
@@ -9468,7 +9468,7 @@
       <c r="B143" s="49" t="s">
         <v>447</v>
       </c>
-      <c r="C143" s="113" t="s">
+      <c r="C143" s="118" t="s">
         <v>293</v>
       </c>
       <c r="D143" s="51" t="s">
@@ -9498,7 +9498,7 @@
       <c r="B144" s="49" t="s">
         <v>295</v>
       </c>
-      <c r="C144" s="114"/>
+      <c r="C144" s="120"/>
       <c r="D144" s="51" t="s">
         <v>410</v>
       </c>
@@ -9623,7 +9623,7 @@
       <c r="B146" s="49" t="s">
         <v>299</v>
       </c>
-      <c r="C146" s="113" t="s">
+      <c r="C146" s="118" t="s">
         <v>337</v>
       </c>
       <c r="D146" s="51" t="s">
@@ -9648,7 +9648,7 @@
       <c r="B147" s="49" t="s">
         <v>301</v>
       </c>
-      <c r="C147" s="115"/>
+      <c r="C147" s="119"/>
       <c r="D147" s="51" t="s">
         <v>413</v>
       </c>
@@ -9671,7 +9671,7 @@
       <c r="B148" s="49" t="s">
         <v>303</v>
       </c>
-      <c r="C148" s="114"/>
+      <c r="C148" s="120"/>
       <c r="D148" s="51" t="s">
         <v>414</v>
       </c>
@@ -10679,7 +10679,7 @@
       <c r="B163" s="49" t="s">
         <v>457</v>
       </c>
-      <c r="C163" s="113" t="s">
+      <c r="C163" s="118" t="s">
         <v>461</v>
       </c>
       <c r="D163" s="51" t="s">
@@ -10711,7 +10711,7 @@
       <c r="B164" s="49" t="s">
         <v>462</v>
       </c>
-      <c r="C164" s="114"/>
+      <c r="C164" s="120"/>
       <c r="D164" s="51" t="s">
         <v>58</v>
       </c>
@@ -11111,6 +11111,16 @@
   </sheetData>
   <autoFilter ref="A2:G169" xr:uid="{6F0F40A8-6867-461F-BBC6-70DC2A7EA672}"/>
   <mergeCells count="25">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="C163:C164"/>
+    <mergeCell ref="C115:C122"/>
+    <mergeCell ref="C125:C128"/>
+    <mergeCell ref="C130:C135"/>
+    <mergeCell ref="C137:C140"/>
+    <mergeCell ref="C143:C144"/>
+    <mergeCell ref="C146:C148"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="E1:G1"/>
@@ -11126,16 +11136,6 @@
     <mergeCell ref="C91:C96"/>
     <mergeCell ref="C98:C99"/>
     <mergeCell ref="C101:C104"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="C163:C164"/>
-    <mergeCell ref="C115:C122"/>
-    <mergeCell ref="C125:C128"/>
-    <mergeCell ref="C130:C135"/>
-    <mergeCell ref="C137:C140"/>
-    <mergeCell ref="C143:C144"/>
-    <mergeCell ref="C146:C148"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -11220,15 +11220,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100CB585F688DEB1347A3B5B5B8C00EFC19" ma:contentTypeVersion="23" ma:contentTypeDescription="Vytvoří nový dokument" ma:contentTypeScope="" ma:versionID="948492b1ee3f456b1d5a5e92045a9601">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xmlns:ns3="26351040-a7a6-4c2d-a8c5-8e82097712a6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="421727d7026b2581477b2034ccb524ed" ns2:_="" ns3:_="">
     <xsd:import namespace="48b746f1-b314-4eb1-99d1-d36e21f31bc3"/>
@@ -11539,6 +11530,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B5C74D-2479-4176-99F4-911FC178577E}">
   <ds:schemaRefs>
@@ -11557,14 +11557,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4530B61-ADC9-483C-96CD-A1E2383A01CC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DBE14C0-4825-4149-9CAA-759AE1E296C2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11581,4 +11573,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4530B61-ADC9-483C-96CD-A1E2383A01CC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update document metadata and enhance workspace configuration
- Adjusted responsibility assignments in multiple documents to accurately reflect roles in the RACI matrices.
- Updated the "02 - Seznam činností" document with new property values for improved clarity and organization.
- Enhanced the workspace configuration to include recent changes in active files and improve navigation through the recently opened files list.
- Streamlined content across various documents to ensure coherence and relevance in the project structure.
</commit_message>
<xml_diff>
--- a/00_Podklady/(šablona) Příloha_1_Matice_informačního_managementu_(RACI).xlsx
+++ b/00_Podklady/(šablona) Příloha_1_Matice_informačního_managementu_(RACI).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liftrock.sharepoint.com/sites/BIMServices/Sdilene dokumenty/General/01_Zakázky/ZAK_2023_060 ŘSD Plzeň CDE koordinátor/knowledge_base/00_Podklady/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="273" documentId="8_{1A589C59-B8ED-4025-8D09-CAE49E68BD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDAFB3EC-F676-40A1-B9DF-2FF7C11FC40B}"/>
+  <xr:revisionPtr revIDLastSave="274" documentId="8_{1A589C59-B8ED-4025-8D09-CAE49E68BD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C56B4A43-69C0-423A-8996-A8B3590FD438}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matice informačního managementu" sheetId="3" r:id="rId1"/>
@@ -1143,9 +1143,6 @@
     <t>Úroveň Rolí</t>
   </si>
   <si>
-    <t>BIM koordinátor Pověřující strany</t>
-  </si>
-  <si>
     <t xml:space="preserve">Správce stavby </t>
   </si>
   <si>
@@ -1483,6 +1480,9 @@
   </si>
   <si>
     <t>Archvování informačních kontejnerů v společném datovém prostředí v souladu s projektovými metodami a postupy pro vytváření informací.</t>
+  </si>
+  <si>
+    <t>Koordinátor BIM</t>
   </si>
 </sst>
 </file>
@@ -2477,11 +2477,26 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="7" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="7" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2502,21 +2517,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="7" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="7" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2869,36 +2869,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:90" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="109" t="s">
         <v>342</v>
       </c>
-      <c r="B1" s="109" t="s">
+      <c r="B1" s="111" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="109" t="s">
+      <c r="C1" s="111" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="109" t="s">
+      <c r="D1" s="111" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="112" t="s">
+      <c r="E1" s="117" t="s">
         <v>349</v>
       </c>
-      <c r="F1" s="113"/>
-      <c r="G1" s="114"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="115" t="s">
+      <c r="F1" s="118"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="120" t="s">
         <v>350</v>
       </c>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="117"/>
-    </row>
-    <row r="2" spans="1:90" s="23" customFormat="1" ht="137.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="122"/>
-      <c r="B2" s="110"/>
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
+      <c r="J1" s="121"/>
+      <c r="K1" s="121"/>
+      <c r="L1" s="122"/>
+    </row>
+    <row r="2" spans="1:90" s="23" customFormat="1" ht="136.80000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="110"/>
+      <c r="B2" s="112"/>
+      <c r="C2" s="112"/>
+      <c r="D2" s="112"/>
       <c r="E2" s="13" t="s">
         <v>336</v>
       </c>
@@ -2908,18 +2908,18 @@
       <c r="G2" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="H2" s="111"/>
+      <c r="H2" s="116"/>
       <c r="I2" s="14" t="s">
+        <v>351</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>464</v>
+      </c>
+      <c r="K2" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="J2" s="15" t="s">
-        <v>351</v>
-      </c>
-      <c r="K2" s="11" t="s">
+      <c r="L2" s="12" t="s">
         <v>353</v>
-      </c>
-      <c r="L2" s="12" t="s">
-        <v>354</v>
       </c>
       <c r="M2" s="22"/>
     </row>
@@ -2928,11 +2928,11 @@
         <v>1</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C3" s="26"/>
       <c r="D3" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E3" s="28" t="s">
         <v>8</v>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="C4" s="38"/>
       <c r="D4" s="39" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E4" s="40" t="s">
         <v>8</v>
@@ -3133,10 +3133,10 @@
         <v>12</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="D5" s="51" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E5" s="52" t="s">
         <v>8</v>
@@ -3168,7 +3168,7 @@
         <v>15</v>
       </c>
       <c r="D6" s="51" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E6" s="52" t="s">
         <v>8</v>
@@ -3200,7 +3200,7 @@
         <v>18</v>
       </c>
       <c r="D7" s="51" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E7" s="52" t="s">
         <v>8</v>
@@ -3230,7 +3230,7 @@
       </c>
       <c r="C8" s="50"/>
       <c r="D8" s="51" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E8" s="52" t="s">
         <v>8</v>
@@ -3260,7 +3260,7 @@
       </c>
       <c r="C9" s="50"/>
       <c r="D9" s="51" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E9" s="52" t="s">
         <v>8</v>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="C10" s="38"/>
       <c r="D10" s="39" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E10" s="40" t="s">
         <v>8</v>
@@ -3396,7 +3396,7 @@
         <v>27</v>
       </c>
       <c r="D11" s="51" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E11" s="52" t="s">
         <v>8</v>
@@ -3428,7 +3428,7 @@
       </c>
       <c r="C12" s="38"/>
       <c r="D12" s="39" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E12" s="40" t="s">
         <v>8</v>
@@ -3529,10 +3529,10 @@
         <v>31</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E13" s="52" t="s">
         <v>8</v>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="C14" s="38"/>
       <c r="D14" s="39" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E14" s="40" t="s">
         <v>8</v>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="C15" s="50"/>
       <c r="D15" s="51" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E15" s="52" t="s">
         <v>8</v>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="C16" s="38"/>
       <c r="D16" s="39" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E16" s="40" t="s">
         <v>8</v>
@@ -3801,10 +3801,10 @@
         <v>39</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D17" s="51" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E17" s="52" t="s">
         <v>8</v>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="C18" s="38"/>
       <c r="D18" s="39" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E18" s="40" t="s">
         <v>8</v>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="C19" s="50"/>
       <c r="D19" s="51" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E19" s="52" t="s">
         <v>8</v>
@@ -3972,7 +3972,7 @@
       </c>
       <c r="C20" s="60"/>
       <c r="D20" s="61" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E20" s="62" t="s">
         <v>8</v>
@@ -4070,11 +4070,11 @@
       <c r="B21" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="118" t="s">
-        <v>430</v>
+      <c r="C21" s="113" t="s">
+        <v>429</v>
       </c>
       <c r="D21" s="51" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E21" s="52" t="s">
         <v>8</v>
@@ -4100,9 +4100,9 @@
       <c r="B22" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="119"/>
+      <c r="C22" s="115"/>
       <c r="D22" s="51" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E22" s="52" t="s">
         <v>8</v>
@@ -4128,9 +4128,9 @@
       <c r="B23" s="49" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="119"/>
+      <c r="C23" s="115"/>
       <c r="D23" s="51" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E23" s="52" t="s">
         <v>8</v>
@@ -4156,9 +4156,9 @@
       <c r="B24" s="49" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="119"/>
+      <c r="C24" s="115"/>
       <c r="D24" s="51" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E24" s="52" t="s">
         <v>8</v>
@@ -4184,9 +4184,9 @@
       <c r="B25" s="49" t="s">
         <v>55</v>
       </c>
-      <c r="C25" s="119"/>
+      <c r="C25" s="115"/>
       <c r="D25" s="51" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E25" s="52" t="s">
         <v>8</v>
@@ -4212,7 +4212,7 @@
       <c r="B26" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="C26" s="120"/>
+      <c r="C26" s="114"/>
       <c r="D26" s="51" t="s">
         <v>58</v>
       </c>
@@ -4242,7 +4242,7 @@
       </c>
       <c r="C27" s="38"/>
       <c r="D27" s="61" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E27" s="40" t="s">
         <v>8</v>
@@ -4345,10 +4345,10 @@
         <v>63</v>
       </c>
       <c r="C28" s="50" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D28" s="51" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E28" s="52" t="s">
         <v>8</v>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="C29" s="72"/>
       <c r="D29" s="73" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E29" s="74" t="s">
         <v>8</v>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="C30" s="38"/>
       <c r="D30" s="39" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E30" s="40" t="s">
         <v>8</v>
@@ -4580,11 +4580,11 @@
       <c r="B31" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="118" t="s">
-        <v>432</v>
+      <c r="C31" s="113" t="s">
+        <v>431</v>
       </c>
       <c r="D31" s="51" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E31" s="52" t="s">
         <v>8</v>
@@ -4612,9 +4612,9 @@
       <c r="B32" s="49" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="119"/>
+      <c r="C32" s="115"/>
       <c r="D32" s="51" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E32" s="52" t="s">
         <v>8</v>
@@ -4642,9 +4642,9 @@
       <c r="B33" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="119"/>
+      <c r="C33" s="115"/>
       <c r="D33" s="51" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E33" s="52" t="s">
         <v>8</v>
@@ -4672,9 +4672,9 @@
       <c r="B34" s="49" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="119"/>
+      <c r="C34" s="115"/>
       <c r="D34" s="51" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E34" s="52" t="s">
         <v>8</v>
@@ -4702,9 +4702,9 @@
       <c r="B35" s="49" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="119"/>
+      <c r="C35" s="115"/>
       <c r="D35" s="51" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E35" s="52" t="s">
         <v>8</v>
@@ -4732,9 +4732,9 @@
       <c r="B36" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="C36" s="120"/>
+      <c r="C36" s="114"/>
       <c r="D36" s="51" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E36" s="52" t="s">
         <v>8</v>
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C37" s="38"/>
       <c r="D37" s="39" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E37" s="40" t="s">
         <v>8</v>
@@ -4866,7 +4866,7 @@
       </c>
       <c r="C38" s="50"/>
       <c r="D38" s="51" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E38" s="52" t="s">
         <v>8</v>
@@ -4898,7 +4898,7 @@
         <v>85</v>
       </c>
       <c r="D39" s="51" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E39" s="52" t="s">
         <v>8</v>
@@ -4927,10 +4927,10 @@
         <v>87</v>
       </c>
       <c r="C40" s="50" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D40" s="51" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E40" s="52" t="s">
         <v>8</v>
@@ -4960,7 +4960,7 @@
       </c>
       <c r="C41" s="38"/>
       <c r="D41" s="61" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E41" s="40" t="s">
         <v>8</v>
@@ -5066,7 +5066,7 @@
         <v>92</v>
       </c>
       <c r="D42" s="51" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E42" s="52" t="s">
         <v>8</v>
@@ -5098,7 +5098,7 @@
       </c>
       <c r="C43" s="50"/>
       <c r="D43" s="51" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E43" s="52" t="s">
         <v>8</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="C44" s="38"/>
       <c r="D44" s="39" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E44" s="40" t="s">
         <v>8</v>
@@ -5230,11 +5230,11 @@
       <c r="B45" s="49" t="s">
         <v>98</v>
       </c>
-      <c r="C45" s="118" t="s">
+      <c r="C45" s="113" t="s">
         <v>99</v>
       </c>
       <c r="D45" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E45" s="52" t="s">
         <v>8</v>
@@ -5262,9 +5262,9 @@
       <c r="B46" s="49" t="s">
         <v>101</v>
       </c>
-      <c r="C46" s="119"/>
+      <c r="C46" s="115"/>
       <c r="D46" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E46" s="52" t="s">
         <v>8</v>
@@ -5292,9 +5292,9 @@
       <c r="B47" s="49" t="s">
         <v>103</v>
       </c>
-      <c r="C47" s="119"/>
+      <c r="C47" s="115"/>
       <c r="D47" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E47" s="52" t="s">
         <v>8</v>
@@ -5322,9 +5322,9 @@
       <c r="B48" s="49" t="s">
         <v>105</v>
       </c>
-      <c r="C48" s="119"/>
+      <c r="C48" s="115"/>
       <c r="D48" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E48" s="52" t="s">
         <v>8</v>
@@ -5352,9 +5352,9 @@
       <c r="B49" s="49" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="119"/>
+      <c r="C49" s="115"/>
       <c r="D49" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E49" s="52" t="s">
         <v>8</v>
@@ -5382,9 +5382,9 @@
       <c r="B50" s="49" t="s">
         <v>109</v>
       </c>
-      <c r="C50" s="119"/>
+      <c r="C50" s="115"/>
       <c r="D50" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E50" s="52" t="s">
         <v>8</v>
@@ -5412,9 +5412,9 @@
       <c r="B51" s="49" t="s">
         <v>111</v>
       </c>
-      <c r="C51" s="119"/>
+      <c r="C51" s="115"/>
       <c r="D51" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E51" s="52" t="s">
         <v>8</v>
@@ -5442,9 +5442,9 @@
       <c r="B52" s="49" t="s">
         <v>113</v>
       </c>
-      <c r="C52" s="119"/>
+      <c r="C52" s="115"/>
       <c r="D52" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E52" s="52" t="s">
         <v>8</v>
@@ -5472,7 +5472,7 @@
       <c r="B53" s="49" t="s">
         <v>115</v>
       </c>
-      <c r="C53" s="120"/>
+      <c r="C53" s="114"/>
       <c r="D53" s="51" t="s">
         <v>58</v>
       </c>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="C54" s="72"/>
       <c r="D54" s="81" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E54" s="74"/>
       <c r="F54" s="75" t="s">
@@ -5606,7 +5606,7 @@
       </c>
       <c r="C55" s="38"/>
       <c r="D55" s="39" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E55" s="40"/>
       <c r="F55" s="41" t="s">
@@ -5705,10 +5705,10 @@
         <v>121</v>
       </c>
       <c r="C56" s="50" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D56" s="51" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E56" s="52"/>
       <c r="F56" s="53" t="s">
@@ -5729,7 +5729,7 @@
       </c>
       <c r="C57" s="50"/>
       <c r="D57" s="51" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E57" s="52"/>
       <c r="F57" s="82" t="s">
@@ -5750,7 +5750,7 @@
       </c>
       <c r="C58" s="50"/>
       <c r="D58" s="51" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E58" s="52"/>
       <c r="F58" s="82" t="s">
@@ -5767,11 +5767,11 @@
         <v>126</v>
       </c>
       <c r="B59" s="37" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C59" s="38"/>
       <c r="D59" s="39" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E59" s="40"/>
       <c r="F59" s="41" t="s">
@@ -5869,13 +5869,13 @@
         <v>127</v>
       </c>
       <c r="B60" s="49" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C60" s="50" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D60" s="51" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E60" s="52"/>
       <c r="F60" s="53" t="s">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="C61" s="38"/>
       <c r="D61" s="39" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E61" s="40"/>
       <c r="F61" s="41"/>
@@ -5994,13 +5994,13 @@
         <v>130</v>
       </c>
       <c r="B62" s="49" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C62" s="50" t="s">
         <v>131</v>
       </c>
       <c r="D62" s="51" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E62" s="52"/>
       <c r="F62" s="53"/>
@@ -6028,7 +6028,7 @@
       </c>
       <c r="C63" s="38"/>
       <c r="D63" s="39" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E63" s="40"/>
       <c r="F63" s="41" t="s">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="C64" s="50"/>
       <c r="D64" s="51" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E64" s="52"/>
       <c r="F64" s="53" t="s">
@@ -6149,7 +6149,7 @@
       </c>
       <c r="C65" s="38"/>
       <c r="D65" s="39" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E65" s="40"/>
       <c r="F65" s="41" t="s">
@@ -6251,7 +6251,7 @@
         <v>140</v>
       </c>
       <c r="D66" s="51" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E66" s="52"/>
       <c r="F66" s="53" t="s">
@@ -6274,7 +6274,7 @@
       </c>
       <c r="C67" s="38"/>
       <c r="D67" s="39" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E67" s="40"/>
       <c r="F67" s="41" t="s">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="C68" s="50"/>
       <c r="D68" s="51" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E68" s="52"/>
       <c r="F68" s="53" t="s">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="C69" s="38"/>
       <c r="D69" s="39" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E69" s="40"/>
       <c r="F69" s="41" t="s">
@@ -6496,13 +6496,13 @@
         <v>148</v>
       </c>
       <c r="B70" s="49" t="s">
-        <v>439</v>
-      </c>
-      <c r="C70" s="118" t="s">
+        <v>438</v>
+      </c>
+      <c r="C70" s="113" t="s">
         <v>149</v>
       </c>
       <c r="D70" s="51" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E70" s="52"/>
       <c r="F70" s="53" t="s">
@@ -6521,9 +6521,9 @@
       <c r="B71" s="49" t="s">
         <v>151</v>
       </c>
-      <c r="C71" s="119"/>
+      <c r="C71" s="115"/>
       <c r="D71" s="51" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E71" s="52"/>
       <c r="F71" s="53" t="s">
@@ -6542,9 +6542,9 @@
       <c r="B72" s="49" t="s">
         <v>153</v>
       </c>
-      <c r="C72" s="119"/>
+      <c r="C72" s="115"/>
       <c r="D72" s="51" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E72" s="52"/>
       <c r="F72" s="53" t="s">
@@ -6563,9 +6563,9 @@
       <c r="B73" s="49" t="s">
         <v>155</v>
       </c>
-      <c r="C73" s="120"/>
+      <c r="C73" s="114"/>
       <c r="D73" s="51" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E73" s="52"/>
       <c r="F73" s="53" t="s">
@@ -6688,7 +6688,7 @@
       <c r="B75" s="49" t="s">
         <v>159</v>
       </c>
-      <c r="C75" s="118" t="s">
+      <c r="C75" s="113" t="s">
         <v>160</v>
       </c>
       <c r="D75" s="51" t="s">
@@ -6722,7 +6722,7 @@
       <c r="B76" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="C76" s="119"/>
+      <c r="C76" s="115"/>
       <c r="D76" s="51" t="s">
         <v>58</v>
       </c>
@@ -6754,7 +6754,7 @@
       <c r="B77" s="49" t="s">
         <v>164</v>
       </c>
-      <c r="C77" s="120"/>
+      <c r="C77" s="114"/>
       <c r="D77" s="51" t="s">
         <v>58</v>
       </c>
@@ -6781,7 +6781,7 @@
       </c>
       <c r="C78" s="72"/>
       <c r="D78" s="81" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E78" s="74" t="s">
         <v>4</v>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="C79" s="38"/>
       <c r="D79" s="39" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E79" s="40" t="s">
         <v>4</v>
@@ -6987,13 +6987,13 @@
         <v>169</v>
       </c>
       <c r="B80" s="49" t="s">
-        <v>440</v>
-      </c>
-      <c r="C80" s="118" t="s">
+        <v>439</v>
+      </c>
+      <c r="C80" s="113" t="s">
         <v>170</v>
       </c>
       <c r="D80" s="51" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E80" s="52" t="s">
         <v>4</v>
@@ -7018,9 +7018,9 @@
       <c r="B81" s="49" t="s">
         <v>172</v>
       </c>
-      <c r="C81" s="119"/>
+      <c r="C81" s="115"/>
       <c r="D81" s="51" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E81" s="52" t="s">
         <v>4</v>
@@ -7045,9 +7045,9 @@
       <c r="B82" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="C82" s="119"/>
+      <c r="C82" s="115"/>
       <c r="D82" s="51" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E82" s="52" t="s">
         <v>4</v>
@@ -7072,9 +7072,9 @@
       <c r="B83" s="49" t="s">
         <v>176</v>
       </c>
-      <c r="C83" s="119"/>
+      <c r="C83" s="115"/>
       <c r="D83" s="51" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E83" s="52" t="s">
         <v>4</v>
@@ -7099,9 +7099,9 @@
       <c r="B84" s="83" t="s">
         <v>178</v>
       </c>
-      <c r="C84" s="119"/>
+      <c r="C84" s="115"/>
       <c r="D84" s="51" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E84" s="52" t="s">
         <v>4</v>
@@ -7126,9 +7126,9 @@
       <c r="B85" s="49" t="s">
         <v>180</v>
       </c>
-      <c r="C85" s="119"/>
+      <c r="C85" s="115"/>
       <c r="D85" s="51" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E85" s="52" t="s">
         <v>4</v>
@@ -7153,9 +7153,9 @@
       <c r="B86" s="49" t="s">
         <v>182</v>
       </c>
-      <c r="C86" s="120"/>
+      <c r="C86" s="114"/>
       <c r="D86" s="51" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="E86" s="52" t="s">
         <v>4</v>
@@ -7182,7 +7182,7 @@
       </c>
       <c r="C87" s="38"/>
       <c r="D87" s="39" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E87" s="40"/>
       <c r="F87" s="41" t="s">
@@ -7282,11 +7282,11 @@
       <c r="B88" s="49" t="s">
         <v>186</v>
       </c>
-      <c r="C88" s="118" t="s">
+      <c r="C88" s="113" t="s">
         <v>187</v>
       </c>
       <c r="D88" s="51" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E88" s="52"/>
       <c r="F88" s="53" t="s">
@@ -7307,7 +7307,7 @@
       <c r="B89" s="49" t="s">
         <v>189</v>
       </c>
-      <c r="C89" s="120"/>
+      <c r="C89" s="114"/>
       <c r="D89" s="51" t="s">
         <v>58</v>
       </c>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="C90" s="38"/>
       <c r="D90" s="39" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E90" s="40"/>
       <c r="F90" s="41" t="s">
@@ -7430,11 +7430,11 @@
       <c r="B91" s="49" t="s">
         <v>191</v>
       </c>
-      <c r="C91" s="118" t="s">
+      <c r="C91" s="113" t="s">
         <v>193</v>
       </c>
       <c r="D91" s="51" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E91" s="84"/>
       <c r="F91" s="53" t="s">
@@ -7453,9 +7453,9 @@
       <c r="B92" s="49" t="s">
         <v>195</v>
       </c>
-      <c r="C92" s="119"/>
+      <c r="C92" s="115"/>
       <c r="D92" s="51" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E92" s="52"/>
       <c r="F92" s="53" t="s">
@@ -7474,9 +7474,9 @@
       <c r="B93" s="49" t="s">
         <v>197</v>
       </c>
-      <c r="C93" s="119"/>
+      <c r="C93" s="115"/>
       <c r="D93" s="51" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E93" s="52"/>
       <c r="F93" s="53" t="s">
@@ -7495,9 +7495,9 @@
       <c r="B94" s="49" t="s">
         <v>199</v>
       </c>
-      <c r="C94" s="119"/>
+      <c r="C94" s="115"/>
       <c r="D94" s="87" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E94" s="52"/>
       <c r="F94" s="53" t="s">
@@ -7516,9 +7516,9 @@
       <c r="B95" s="49" t="s">
         <v>201</v>
       </c>
-      <c r="C95" s="119"/>
+      <c r="C95" s="115"/>
       <c r="D95" s="87" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E95" s="52"/>
       <c r="F95" s="53" t="s">
@@ -7537,9 +7537,9 @@
       <c r="B96" s="49" t="s">
         <v>203</v>
       </c>
-      <c r="C96" s="120"/>
+      <c r="C96" s="114"/>
       <c r="D96" s="87" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E96" s="52"/>
       <c r="F96" s="53" t="s">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="C97" s="38"/>
       <c r="D97" s="39" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E97" s="40"/>
       <c r="F97" s="41" t="s">
@@ -7660,7 +7660,7 @@
       <c r="B98" s="49" t="s">
         <v>207</v>
       </c>
-      <c r="C98" s="118" t="s">
+      <c r="C98" s="113" t="s">
         <v>208</v>
       </c>
       <c r="D98" s="51" t="s">
@@ -7683,9 +7683,9 @@
       <c r="B99" s="49" t="s">
         <v>210</v>
       </c>
-      <c r="C99" s="120"/>
+      <c r="C99" s="114"/>
       <c r="D99" s="51" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E99" s="52"/>
       <c r="F99" s="53" t="s">
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C100" s="38"/>
       <c r="D100" s="39" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E100" s="40" t="s">
         <v>4</v>
@@ -7810,11 +7810,11 @@
       <c r="B101" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="C101" s="118" t="s">
+      <c r="C101" s="113" t="s">
         <v>216</v>
       </c>
       <c r="D101" s="51" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E101" s="84"/>
       <c r="F101" s="53" t="s">
@@ -7835,9 +7835,9 @@
       <c r="B102" s="49" t="s">
         <v>218</v>
       </c>
-      <c r="C102" s="119"/>
+      <c r="C102" s="115"/>
       <c r="D102" s="51" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E102" s="52"/>
       <c r="F102" s="53" t="s">
@@ -7858,9 +7858,9 @@
       <c r="B103" s="49" t="s">
         <v>220</v>
       </c>
-      <c r="C103" s="119"/>
+      <c r="C103" s="115"/>
       <c r="D103" s="51" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E103" s="52"/>
       <c r="F103" s="53" t="s">
@@ -7881,9 +7881,9 @@
       <c r="B104" s="49" t="s">
         <v>222</v>
       </c>
-      <c r="C104" s="120"/>
+      <c r="C104" s="114"/>
       <c r="D104" s="51" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E104" s="52" t="s">
         <v>4</v>
@@ -7910,7 +7910,7 @@
       </c>
       <c r="C105" s="38"/>
       <c r="D105" s="39" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E105" s="40" t="s">
         <v>8</v>
@@ -8012,11 +8012,11 @@
       <c r="B106" s="49" t="s">
         <v>226</v>
       </c>
-      <c r="C106" s="118" t="s">
-        <v>443</v>
+      <c r="C106" s="113" t="s">
+        <v>442</v>
       </c>
       <c r="D106" s="51" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E106" s="84" t="s">
         <v>8</v>
@@ -8039,9 +8039,9 @@
       <c r="B107" s="49" t="s">
         <v>228</v>
       </c>
-      <c r="C107" s="119"/>
+      <c r="C107" s="115"/>
       <c r="D107" s="51" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E107" s="84" t="s">
         <v>8</v>
@@ -8064,9 +8064,9 @@
       <c r="B108" s="49" t="s">
         <v>230</v>
       </c>
-      <c r="C108" s="119"/>
+      <c r="C108" s="115"/>
       <c r="D108" s="51" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E108" s="84" t="s">
         <v>8</v>
@@ -8089,9 +8089,9 @@
       <c r="B109" s="49" t="s">
         <v>232</v>
       </c>
-      <c r="C109" s="119"/>
+      <c r="C109" s="115"/>
       <c r="D109" s="51" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E109" s="84" t="s">
         <v>8</v>
@@ -8112,11 +8112,11 @@
         <v>233</v>
       </c>
       <c r="B110" s="49" t="s">
-        <v>441</v>
-      </c>
-      <c r="C110" s="119"/>
+        <v>440</v>
+      </c>
+      <c r="C110" s="115"/>
       <c r="D110" s="51" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E110" s="84" t="s">
         <v>8</v>
@@ -8139,9 +8139,9 @@
       <c r="B111" s="49" t="s">
         <v>235</v>
       </c>
-      <c r="C111" s="119"/>
+      <c r="C111" s="115"/>
       <c r="D111" s="51" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E111" s="84" t="s">
         <v>8</v>
@@ -8162,9 +8162,9 @@
         <v>236</v>
       </c>
       <c r="B112" s="49" t="s">
-        <v>442</v>
-      </c>
-      <c r="C112" s="119"/>
+        <v>441</v>
+      </c>
+      <c r="C112" s="115"/>
       <c r="D112" s="51" t="s">
         <v>58</v>
       </c>
@@ -8189,7 +8189,7 @@
       <c r="B113" s="49" t="s">
         <v>238</v>
       </c>
-      <c r="C113" s="120"/>
+      <c r="C113" s="114"/>
       <c r="D113" s="51" t="s">
         <v>58</v>
       </c>
@@ -8216,7 +8216,7 @@
       </c>
       <c r="C114" s="38"/>
       <c r="D114" s="39" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E114" s="40"/>
       <c r="F114" s="41" t="s">
@@ -8316,11 +8316,11 @@
       <c r="B115" s="49" t="s">
         <v>242</v>
       </c>
-      <c r="C115" s="118" t="s">
-        <v>444</v>
+      <c r="C115" s="113" t="s">
+        <v>443</v>
       </c>
       <c r="D115" s="51" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E115" s="84"/>
       <c r="F115" s="53" t="s">
@@ -8334,16 +8334,16 @@
       <c r="K115" s="53"/>
       <c r="L115" s="57"/>
     </row>
-    <row r="116" spans="1:90" ht="26.4" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:90" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A116" s="48" t="s">
         <v>243</v>
       </c>
       <c r="B116" s="49" t="s">
         <v>244</v>
       </c>
-      <c r="C116" s="119"/>
+      <c r="C116" s="115"/>
       <c r="D116" s="51" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E116" s="84"/>
       <c r="F116" s="53" t="s">
@@ -8364,9 +8364,9 @@
       <c r="B117" s="49" t="s">
         <v>230</v>
       </c>
-      <c r="C117" s="119"/>
+      <c r="C117" s="115"/>
       <c r="D117" s="51" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E117" s="84"/>
       <c r="F117" s="53" t="s">
@@ -8387,9 +8387,9 @@
       <c r="B118" s="49" t="s">
         <v>232</v>
       </c>
-      <c r="C118" s="119"/>
+      <c r="C118" s="115"/>
       <c r="D118" s="51" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E118" s="84"/>
       <c r="F118" s="53" t="s">
@@ -8408,11 +8408,11 @@
         <v>247</v>
       </c>
       <c r="B119" s="49" t="s">
-        <v>441</v>
-      </c>
-      <c r="C119" s="119"/>
+        <v>440</v>
+      </c>
+      <c r="C119" s="115"/>
       <c r="D119" s="51" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E119" s="84"/>
       <c r="F119" s="53" t="s">
@@ -8433,9 +8433,9 @@
       <c r="B120" s="49" t="s">
         <v>249</v>
       </c>
-      <c r="C120" s="119"/>
+      <c r="C120" s="115"/>
       <c r="D120" s="51" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E120" s="84"/>
       <c r="F120" s="53" t="s">
@@ -8454,9 +8454,9 @@
         <v>250</v>
       </c>
       <c r="B121" s="49" t="s">
-        <v>442</v>
-      </c>
-      <c r="C121" s="119"/>
+        <v>441</v>
+      </c>
+      <c r="C121" s="115"/>
       <c r="D121" s="51" t="s">
         <v>58</v>
       </c>
@@ -8479,7 +8479,7 @@
       <c r="B122" s="49" t="s">
         <v>252</v>
       </c>
-      <c r="C122" s="120"/>
+      <c r="C122" s="114"/>
       <c r="D122" s="51" t="s">
         <v>58</v>
       </c>
@@ -8504,7 +8504,7 @@
       </c>
       <c r="C123" s="72"/>
       <c r="D123" s="81" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E123" s="74"/>
       <c r="F123" s="75" t="s">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="C124" s="38"/>
       <c r="D124" s="39" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E124" s="40"/>
       <c r="F124" s="41" t="s">
@@ -8706,11 +8706,11 @@
       <c r="B125" s="49" t="s">
         <v>257</v>
       </c>
-      <c r="C125" s="118" t="s">
+      <c r="C125" s="113" t="s">
         <v>258</v>
       </c>
       <c r="D125" s="51" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E125" s="84"/>
       <c r="F125" s="53" t="s">
@@ -8731,9 +8731,9 @@
       <c r="B126" s="49" t="s">
         <v>260</v>
       </c>
-      <c r="C126" s="119"/>
+      <c r="C126" s="115"/>
       <c r="D126" s="51" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E126" s="84"/>
       <c r="F126" s="53" t="s">
@@ -8754,9 +8754,9 @@
       <c r="B127" s="49" t="s">
         <v>262</v>
       </c>
-      <c r="C127" s="119"/>
+      <c r="C127" s="115"/>
       <c r="D127" s="51" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E127" s="84"/>
       <c r="F127" s="53" t="s">
@@ -8777,9 +8777,9 @@
       <c r="B128" s="49" t="s">
         <v>264</v>
       </c>
-      <c r="C128" s="120"/>
+      <c r="C128" s="114"/>
       <c r="D128" s="51" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E128" s="84"/>
       <c r="F128" s="53" t="s">
@@ -8802,7 +8802,7 @@
       </c>
       <c r="C129" s="38"/>
       <c r="D129" s="39" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E129" s="40"/>
       <c r="F129" s="41" t="s">
@@ -8902,11 +8902,11 @@
       <c r="B130" s="49" t="s">
         <v>268</v>
       </c>
-      <c r="C130" s="118" t="s">
+      <c r="C130" s="113" t="s">
         <v>269</v>
       </c>
       <c r="D130" s="51" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E130" s="84" t="s">
         <v>1</v>
@@ -8929,9 +8929,9 @@
       <c r="B131" s="49" t="s">
         <v>271</v>
       </c>
-      <c r="C131" s="119"/>
+      <c r="C131" s="115"/>
       <c r="D131" s="51" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E131" s="84" t="s">
         <v>1</v>
@@ -8952,11 +8952,11 @@
         <v>272</v>
       </c>
       <c r="B132" s="49" t="s">
-        <v>445</v>
-      </c>
-      <c r="C132" s="119"/>
+        <v>444</v>
+      </c>
+      <c r="C132" s="115"/>
       <c r="D132" s="51" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E132" s="84" t="s">
         <v>1</v>
@@ -8977,11 +8977,11 @@
         <v>273</v>
       </c>
       <c r="B133" s="49" t="s">
-        <v>446</v>
-      </c>
-      <c r="C133" s="119"/>
+        <v>445</v>
+      </c>
+      <c r="C133" s="115"/>
       <c r="D133" s="51" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E133" s="84" t="s">
         <v>4</v>
@@ -9004,9 +9004,9 @@
       <c r="B134" s="49" t="s">
         <v>275</v>
       </c>
-      <c r="C134" s="119"/>
+      <c r="C134" s="115"/>
       <c r="D134" s="51" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E134" s="84" t="s">
         <v>1</v>
@@ -9029,9 +9029,9 @@
       <c r="B135" s="49" t="s">
         <v>277</v>
       </c>
-      <c r="C135" s="120"/>
+      <c r="C135" s="114"/>
       <c r="D135" s="51" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E135" s="84" t="s">
         <v>1</v>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C136" s="38"/>
       <c r="D136" s="39" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E136" s="40" t="s">
         <v>4</v>
@@ -9160,11 +9160,11 @@
       <c r="B137" s="49" t="s">
         <v>281</v>
       </c>
-      <c r="C137" s="118" t="s">
+      <c r="C137" s="113" t="s">
         <v>282</v>
       </c>
       <c r="D137" s="51" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E137" s="84" t="s">
         <v>4</v>
@@ -9189,9 +9189,9 @@
       <c r="B138" s="49" t="s">
         <v>284</v>
       </c>
-      <c r="C138" s="119"/>
+      <c r="C138" s="115"/>
       <c r="D138" s="51" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E138" s="84"/>
       <c r="F138" s="53" t="s">
@@ -9214,9 +9214,9 @@
       <c r="B139" s="49" t="s">
         <v>286</v>
       </c>
-      <c r="C139" s="119"/>
+      <c r="C139" s="115"/>
       <c r="D139" s="51" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E139" s="84"/>
       <c r="F139" s="53" t="s">
@@ -9239,9 +9239,9 @@
       <c r="B140" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C140" s="120"/>
+      <c r="C140" s="114"/>
       <c r="D140" s="51" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E140" s="84"/>
       <c r="F140" s="53" t="s">
@@ -9266,7 +9266,7 @@
       </c>
       <c r="C141" s="72"/>
       <c r="D141" s="81" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E141" s="74"/>
       <c r="F141" s="75" t="s">
@@ -9368,7 +9368,7 @@
       </c>
       <c r="C142" s="38"/>
       <c r="D142" s="39" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E142" s="40"/>
       <c r="F142" s="41" t="s">
@@ -9466,13 +9466,13 @@
         <v>292</v>
       </c>
       <c r="B143" s="49" t="s">
-        <v>447</v>
-      </c>
-      <c r="C143" s="118" t="s">
+        <v>446</v>
+      </c>
+      <c r="C143" s="113" t="s">
         <v>293</v>
       </c>
       <c r="D143" s="51" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E143" s="84"/>
       <c r="F143" s="53"/>
@@ -9498,9 +9498,9 @@
       <c r="B144" s="49" t="s">
         <v>295</v>
       </c>
-      <c r="C144" s="120"/>
+      <c r="C144" s="114"/>
       <c r="D144" s="51" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E144" s="84"/>
       <c r="F144" s="53" t="s">
@@ -9523,7 +9523,7 @@
       </c>
       <c r="C145" s="38"/>
       <c r="D145" s="39" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E145" s="40"/>
       <c r="F145" s="41" t="s">
@@ -9623,11 +9623,11 @@
       <c r="B146" s="49" t="s">
         <v>299</v>
       </c>
-      <c r="C146" s="118" t="s">
+      <c r="C146" s="113" t="s">
         <v>337</v>
       </c>
       <c r="D146" s="51" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E146" s="84"/>
       <c r="F146" s="53" t="s">
@@ -9648,9 +9648,9 @@
       <c r="B147" s="49" t="s">
         <v>301</v>
       </c>
-      <c r="C147" s="119"/>
+      <c r="C147" s="115"/>
       <c r="D147" s="51" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E147" s="84"/>
       <c r="F147" s="53" t="s">
@@ -9671,9 +9671,9 @@
       <c r="B148" s="49" t="s">
         <v>303</v>
       </c>
-      <c r="C148" s="120"/>
+      <c r="C148" s="114"/>
       <c r="D148" s="51" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E148" s="84"/>
       <c r="F148" s="53" t="s">
@@ -9696,7 +9696,7 @@
       </c>
       <c r="C149" s="38"/>
       <c r="D149" s="39" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E149" s="40"/>
       <c r="F149" s="41" t="s">
@@ -9797,10 +9797,10 @@
         <v>307</v>
       </c>
       <c r="C150" s="50" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D150" s="51" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E150" s="84"/>
       <c r="F150" s="53" t="s">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="C151" s="38"/>
       <c r="D151" s="39" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E151" s="40"/>
       <c r="F151" s="41" t="s">
@@ -9924,10 +9924,10 @@
         <v>311</v>
       </c>
       <c r="C152" s="50" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="D152" s="51" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E152" s="84"/>
       <c r="F152" s="53" t="s">
@@ -9946,11 +9946,11 @@
         <v>312</v>
       </c>
       <c r="B153" s="37" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C153" s="38"/>
       <c r="D153" s="39" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E153" s="40"/>
       <c r="F153" s="41" t="s">
@@ -10048,13 +10048,13 @@
         <v>313</v>
       </c>
       <c r="B154" s="49" t="s">
+        <v>448</v>
+      </c>
+      <c r="C154" s="50" t="s">
         <v>449</v>
       </c>
-      <c r="C154" s="50" t="s">
-        <v>450</v>
-      </c>
       <c r="D154" s="51" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E154" s="84"/>
       <c r="F154" s="53" t="s">
@@ -10073,11 +10073,11 @@
         <v>7</v>
       </c>
       <c r="B155" s="71" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C155" s="72"/>
       <c r="D155" s="81" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E155" s="74" t="s">
         <v>314</v>
@@ -10181,7 +10181,7 @@
       </c>
       <c r="C156" s="38"/>
       <c r="D156" s="39" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E156" s="40"/>
       <c r="F156" s="41" t="s">
@@ -10282,10 +10282,10 @@
         <v>318</v>
       </c>
       <c r="C157" s="50" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D157" s="51" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E157" s="84"/>
       <c r="F157" s="53" t="s">
@@ -10304,11 +10304,11 @@
         <v>319</v>
       </c>
       <c r="B158" s="37" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C158" s="38"/>
       <c r="D158" s="39" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E158" s="40"/>
       <c r="F158" s="41" t="s">
@@ -10409,10 +10409,10 @@
         <v>321</v>
       </c>
       <c r="C159" s="50" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D159" s="51" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E159" s="84"/>
       <c r="F159" s="53" t="s">
@@ -10431,11 +10431,11 @@
         <v>322</v>
       </c>
       <c r="B160" s="37" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C160" s="38"/>
       <c r="D160" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E160" s="40" t="s">
         <v>4</v>
@@ -10538,10 +10538,10 @@
         <v>324</v>
       </c>
       <c r="C161" s="50" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="D161" s="51" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E161" s="84" t="s">
         <v>4</v>
@@ -10571,11 +10571,11 @@
         <v>325</v>
       </c>
       <c r="B162" s="37" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C162" s="38"/>
       <c r="D162" s="39" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E162" s="40" t="s">
         <v>8</v>
@@ -10677,13 +10677,13 @@
         <v>326</v>
       </c>
       <c r="B163" s="49" t="s">
-        <v>457</v>
-      </c>
-      <c r="C163" s="118" t="s">
-        <v>461</v>
+        <v>456</v>
+      </c>
+      <c r="C163" s="113" t="s">
+        <v>460</v>
       </c>
       <c r="D163" s="51" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E163" s="84" t="s">
         <v>8</v>
@@ -10709,9 +10709,9 @@
         <v>327</v>
       </c>
       <c r="B164" s="49" t="s">
-        <v>462</v>
-      </c>
-      <c r="C164" s="120"/>
+        <v>461</v>
+      </c>
+      <c r="C164" s="114"/>
       <c r="D164" s="51" t="s">
         <v>58</v>
       </c>
@@ -10740,7 +10740,7 @@
       </c>
       <c r="C165" s="72"/>
       <c r="D165" s="81" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E165" s="74" t="s">
         <v>8</v>
@@ -10840,11 +10840,11 @@
         <v>329</v>
       </c>
       <c r="B166" s="37" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C166" s="38"/>
       <c r="D166" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E166" s="40" t="s">
         <v>8</v>
@@ -10942,13 +10942,13 @@
         <v>330</v>
       </c>
       <c r="B167" s="49" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C167" s="50" t="s">
         <v>331</v>
       </c>
       <c r="D167" s="51" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E167" s="84" t="s">
         <v>8</v>
@@ -10978,7 +10978,7 @@
       </c>
       <c r="C168" s="90"/>
       <c r="D168" s="91" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E168" s="92" t="s">
         <v>8</v>
@@ -11084,7 +11084,7 @@
       </c>
       <c r="C169" s="108"/>
       <c r="D169" s="97" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E169" s="98" t="s">
         <v>8</v>
@@ -11111,16 +11111,6 @@
   </sheetData>
   <autoFilter ref="A2:G169" xr:uid="{6F0F40A8-6867-461F-BBC6-70DC2A7EA672}"/>
   <mergeCells count="25">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="C163:C164"/>
-    <mergeCell ref="C115:C122"/>
-    <mergeCell ref="C125:C128"/>
-    <mergeCell ref="C130:C135"/>
-    <mergeCell ref="C137:C140"/>
-    <mergeCell ref="C143:C144"/>
-    <mergeCell ref="C146:C148"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="E1:G1"/>
@@ -11136,6 +11126,16 @@
     <mergeCell ref="C91:C96"/>
     <mergeCell ref="C98:C99"/>
     <mergeCell ref="C101:C104"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="C163:C164"/>
+    <mergeCell ref="C115:C122"/>
+    <mergeCell ref="C125:C128"/>
+    <mergeCell ref="C130:C135"/>
+    <mergeCell ref="C137:C140"/>
+    <mergeCell ref="C143:C144"/>
+    <mergeCell ref="C146:C148"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -11220,6 +11220,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100CB585F688DEB1347A3B5B5B8C00EFC19" ma:contentTypeVersion="23" ma:contentTypeDescription="Vytvoří nový dokument" ma:contentTypeScope="" ma:versionID="948492b1ee3f456b1d5a5e92045a9601">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xmlns:ns3="26351040-a7a6-4c2d-a8c5-8e82097712a6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="421727d7026b2581477b2034ccb524ed" ns2:_="" ns3:_="">
     <xsd:import namespace="48b746f1-b314-4eb1-99d1-d36e21f31bc3"/>
@@ -11530,15 +11539,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B5C74D-2479-4176-99F4-911FC178577E}">
   <ds:schemaRefs>
@@ -11557,6 +11557,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4530B61-ADC9-483C-96CD-A1E2383A01CC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DBE14C0-4825-4149-9CAA-759AE1E296C2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11573,12 +11581,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4530B61-ADC9-483C-96CD-A1E2383A01CC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>